<commit_message>
Stock report conversion fix, Manual Top Up Report for LINTEAM
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="11"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -877,9 +877,6 @@
     <t>Rental Hygiene</t>
   </si>
   <si>
-    <t>1/12</t>
-  </si>
-  <si>
     <t>CSG/Jeff Supplies</t>
   </si>
   <si>
@@ -945,6 +942,9 @@
   <si>
     <t>WIPY KLEEN-AP60
 (Kohe)</t>
+  </si>
+  <si>
+    <t>1/12</t>
   </si>
   <si>
     <t>3M</t>
@@ -4994,7 +4994,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5019,9 +5019,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -73891,7 +73888,7 @@
     <col min="1" max="2" width="44.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>261</v>
       </c>
@@ -73899,7 +73896,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="2" ht="14.5">
+    <row r="2">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -73907,7 +73904,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="3" ht="14.5">
+    <row r="3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -73915,7 +73912,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="4" ht="14.5">
+    <row r="4">
       <c r="A4" t="s">
         <v>152</v>
       </c>
@@ -73923,13 +73920,13 @@
         <v>152</v>
       </c>
     </row>
-    <row r="5" ht="14.5">
+    <row r="5">
       <c r="A5"/>
       <c r="B5" s="3" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="6" ht="14.5">
+    <row r="6">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -73937,7 +73934,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="7" ht="14.5">
+    <row r="7">
       <c r="A7" t="s">
         <v>97</v>
       </c>
@@ -73945,7 +73942,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="8" ht="14.5">
+    <row r="8">
       <c r="A8" t="s">
         <v>153</v>
       </c>
@@ -73953,7 +73950,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="9" ht="14.5">
+    <row r="9">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -73961,7 +73958,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="10" ht="14.5">
+    <row r="10">
       <c r="A10" t="s">
         <v>50</v>
       </c>
@@ -73969,7 +73966,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="11" ht="14.5">
+    <row r="11">
       <c r="A11" t="s">
         <v>262</v>
       </c>
@@ -73977,7 +73974,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="12" ht="14.5">
+    <row r="12">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -73985,7 +73982,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" ht="14.5">
+    <row r="13">
       <c r="A13" t="s">
         <v>92</v>
       </c>
@@ -73993,7 +73990,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" ht="14.5">
+    <row r="14">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -74001,7 +73998,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="15" ht="14.5">
+    <row r="15">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -74009,7 +74006,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="16" ht="14.5">
+    <row r="16">
       <c r="A16" t="s">
         <v>147</v>
       </c>
@@ -74017,7 +74014,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="17" ht="14.5">
+    <row r="17">
       <c r="A17" t="s">
         <v>148</v>
       </c>
@@ -74025,7 +74022,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="18" ht="14.5">
+    <row r="18">
       <c r="A18" t="s">
         <v>149</v>
       </c>
@@ -74033,7 +74030,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="19" ht="14.5">
+    <row r="19">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -74041,7 +74038,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="20" ht="14.5">
+    <row r="20">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -74049,7 +74046,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="21" ht="14.5">
+    <row r="21">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -74057,7 +74054,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="22" ht="14.5">
+    <row r="22">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -74065,7 +74062,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="23" ht="14.5">
+    <row r="23">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -74073,7 +74070,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" ht="14.5">
+    <row r="24">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -74081,7 +74078,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="25" ht="14.5">
+    <row r="25">
       <c r="A25" t="s">
         <v>54</v>
       </c>
@@ -74089,7 +74086,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="26" ht="14.5">
+    <row r="26">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -74097,7 +74094,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="27" ht="14.5">
+    <row r="27">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -74105,7 +74102,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="28" ht="14.5">
+    <row r="28">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -74113,7 +74110,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="29" ht="14.5">
+    <row r="29">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -74121,7 +74118,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="30" ht="14.5">
+    <row r="30">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -74129,7 +74126,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="31" ht="14.5">
+    <row r="31">
       <c r="A31" t="s">
         <v>55</v>
       </c>
@@ -74137,7 +74134,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="32" ht="14.5">
+    <row r="32">
       <c r="A32" t="s">
         <v>135</v>
       </c>
@@ -74145,7 +74142,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="33" ht="14.5">
+    <row r="33">
       <c r="A33" t="s">
         <v>129</v>
       </c>
@@ -74153,7 +74150,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="34" ht="14.5">
+    <row r="34">
       <c r="A34" t="s">
         <v>127</v>
       </c>
@@ -74161,7 +74158,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="35" ht="14.5">
+    <row r="35">
       <c r="A35" t="s">
         <v>128</v>
       </c>
@@ -74169,7 +74166,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="36" ht="14.5">
+    <row r="36">
       <c r="A36" t="s">
         <v>107</v>
       </c>
@@ -74177,7 +74174,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="37" ht="14.5">
+    <row r="37">
       <c r="A37" t="s">
         <v>83</v>
       </c>
@@ -74185,7 +74182,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="38" ht="14.5">
+    <row r="38">
       <c r="A38" t="s">
         <v>155</v>
       </c>
@@ -74193,7 +74190,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="39" ht="14.5">
+    <row r="39">
       <c r="A39" t="s">
         <v>156</v>
       </c>
@@ -74201,7 +74198,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="40" ht="14.5">
+    <row r="40">
       <c r="A40" t="s">
         <v>119</v>
       </c>
@@ -74209,7 +74206,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="41" ht="14.5">
+    <row r="41">
       <c r="A41" t="s">
         <v>120</v>
       </c>
@@ -74217,7 +74214,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="42" ht="14.5">
+    <row r="42">
       <c r="A42" t="s">
         <v>143</v>
       </c>
@@ -74225,7 +74222,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="43" ht="14.5">
+    <row r="43">
       <c r="A43" t="s">
         <v>144</v>
       </c>
@@ -74233,7 +74230,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="44" ht="14.5">
+    <row r="44">
       <c r="A44" t="s">
         <v>145</v>
       </c>
@@ -74241,7 +74238,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="45" ht="14.5">
+    <row r="45">
       <c r="A45" t="s">
         <v>146</v>
       </c>
@@ -74249,7 +74246,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="46" ht="14.5">
+    <row r="46">
       <c r="A46" t="s">
         <v>84</v>
       </c>
@@ -74257,7 +74254,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="47" ht="14.5">
+    <row r="47">
       <c r="A47" t="s">
         <v>130</v>
       </c>
@@ -74265,7 +74262,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="48" ht="14.5">
+    <row r="48">
       <c r="A48" t="s">
         <v>131</v>
       </c>
@@ -74273,7 +74270,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="49" ht="14.5">
+    <row r="49">
       <c r="A49" t="s">
         <v>114</v>
       </c>
@@ -74281,7 +74278,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="50" ht="14.5">
+    <row r="50">
       <c r="A50" t="s">
         <v>132</v>
       </c>
@@ -74289,7 +74286,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="51" ht="14.5">
+    <row r="51">
       <c r="A51" t="s">
         <v>157</v>
       </c>
@@ -74297,7 +74294,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="52" ht="14.5">
+    <row r="52">
       <c r="A52" t="s">
         <v>108</v>
       </c>
@@ -74305,7 +74302,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="53" ht="14.5">
+    <row r="53">
       <c r="A53" t="s">
         <v>154</v>
       </c>
@@ -74313,7 +74310,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="54" ht="14.5">
+    <row r="54">
       <c r="A54" t="s">
         <v>105</v>
       </c>
@@ -74321,7 +74318,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="55" ht="14.5">
+    <row r="55">
       <c r="A55" t="s">
         <v>106</v>
       </c>
@@ -74329,7 +74326,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="56" ht="14.5">
+    <row r="56">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -74337,7 +74334,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="57" ht="14.5">
+    <row r="57">
       <c r="A57" t="s">
         <v>122</v>
       </c>
@@ -74345,7 +74342,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="58" ht="14.5">
+    <row r="58">
       <c r="A58" t="s">
         <v>158</v>
       </c>
@@ -74353,7 +74350,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="59" ht="14.5">
+    <row r="59">
       <c r="A59" t="s">
         <v>57</v>
       </c>
@@ -74361,7 +74358,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="60" ht="14.5">
+    <row r="60">
       <c r="A60" t="s">
         <v>64</v>
       </c>
@@ -74369,7 +74366,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="61" ht="14.5">
+    <row r="61">
       <c r="A61" t="s">
         <v>139</v>
       </c>
@@ -74377,7 +74374,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="62" ht="14.5">
+    <row r="62">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -74385,7 +74382,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="63" ht="14.5">
+    <row r="63">
       <c r="A63" t="s">
         <v>61</v>
       </c>
@@ -74393,7 +74390,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="64" ht="14.5">
+    <row r="64">
       <c r="A64" t="s">
         <v>72</v>
       </c>
@@ -74401,7 +74398,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="65" ht="14.5">
+    <row r="65">
       <c r="A65" t="s">
         <v>159</v>
       </c>
@@ -74409,7 +74406,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="66" ht="14.5">
+    <row r="66">
       <c r="A66" t="s">
         <v>140</v>
       </c>
@@ -74417,7 +74414,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="67" ht="14.5">
+    <row r="67">
       <c r="A67" t="s">
         <v>74</v>
       </c>
@@ -74425,7 +74422,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="68" ht="14.5">
+    <row r="68">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -74433,12 +74430,12 @@
         <v>256</v>
       </c>
     </row>
-    <row r="69" ht="14.5">
+    <row r="69">
       <c r="B69" s="3" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="70" ht="14.5">
+    <row r="70">
       <c r="A70" t="s">
         <v>160</v>
       </c>
@@ -74446,12 +74443,12 @@
         <v>160</v>
       </c>
     </row>
-    <row r="71" ht="14.5">
+    <row r="71">
       <c r="B71" s="3" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="72" ht="14.5">
+    <row r="72">
       <c r="A72" t="s">
         <v>166</v>
       </c>
@@ -74759,8 +74756,8 @@
       <c r="H9" s="8">
         <v>32.700000000000003</v>
       </c>
-      <c r="I9" s="10" t="s">
-        <v>280</v>
+      <c r="I9" s="9">
+        <v>1</v>
       </c>
       <c r="J9" s="5" t="s">
         <v>15</v>
@@ -74780,7 +74777,7 @@
         <v>179</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>184</v>
@@ -74812,7 +74809,7 @@
         <v>179</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>184</v>
@@ -74835,7 +74832,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>35</v>
@@ -74844,7 +74841,7 @@
         <v>179</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>178</v>
@@ -74867,7 +74864,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>30</v>
@@ -74876,7 +74873,7 @@
         <v>179</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>178</v>
@@ -74899,7 +74896,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>262</v>
@@ -74908,7 +74905,7 @@
         <v>179</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>178</v>
@@ -74931,7 +74928,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>27</v>
@@ -74940,7 +74937,7 @@
         <v>179</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F15" s="5" t="s">
         <v>178</v>
@@ -74963,7 +74960,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>34</v>
@@ -74972,7 +74969,7 @@
         <v>179</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F16" s="5" t="s">
         <v>178</v>
@@ -74995,7 +74992,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>33</v>
@@ -75004,7 +75001,7 @@
         <v>179</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>178</v>
@@ -75027,7 +75024,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>32</v>
@@ -75036,7 +75033,7 @@
         <v>179</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>178</v>
@@ -75059,7 +75056,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>52</v>
@@ -75068,7 +75065,7 @@
         <v>179</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>178</v>
@@ -75091,7 +75088,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>54</v>
@@ -75100,7 +75097,7 @@
         <v>179</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>178</v>
@@ -75132,7 +75129,7 @@
         <v>179</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>192</v>
@@ -75155,7 +75152,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>49</v>
@@ -75164,7 +75161,7 @@
         <v>179</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>192</v>
@@ -75187,7 +75184,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>50</v>
@@ -75196,7 +75193,7 @@
         <v>179</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>192</v>
@@ -75219,7 +75216,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>51</v>
@@ -75228,7 +75225,7 @@
         <v>179</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>192</v>
@@ -75260,7 +75257,7 @@
         <v>179</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>184</v>
@@ -75292,7 +75289,7 @@
         <v>179</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>182</v>
@@ -75304,7 +75301,7 @@
         <v>60.369999999999997</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>15</v>
@@ -75324,7 +75321,7 @@
         <v>179</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F27" s="5" t="s">
         <v>190</v>
@@ -75450,7 +75447,7 @@
         <v>179</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>178</v>
@@ -75482,7 +75479,7 @@
         <v>225</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>178</v>
@@ -75514,7 +75511,7 @@
         <v>225</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>184</v>
@@ -75546,7 +75543,7 @@
         <v>225</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>89</v>
@@ -75578,7 +75575,7 @@
         <v>225</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>184</v>
@@ -75610,7 +75607,7 @@
         <v>225</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>184</v>
@@ -75642,7 +75639,7 @@
         <v>225</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>184</v>
@@ -75674,7 +75671,7 @@
         <v>225</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>184</v>
@@ -75706,7 +75703,7 @@
         <v>225</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F39" s="5" t="s">
         <v>184</v>
@@ -75768,7 +75765,7 @@
         <v>225</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F41" s="5" t="s">
         <v>184</v>
@@ -75800,7 +75797,7 @@
         <v>225</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F42" s="5" t="s">
         <v>184</v>
@@ -75832,7 +75829,7 @@
         <v>225</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F43" s="5" t="s">
         <v>184</v>
@@ -75864,7 +75861,7 @@
         <v>225</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F44" s="5" t="s">
         <v>184</v>
@@ -75896,7 +75893,7 @@
         <v>225</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>184</v>
@@ -75928,7 +75925,7 @@
         <v>225</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>184</v>
@@ -75960,7 +75957,7 @@
         <v>225</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F47" s="5" t="s">
         <v>184</v>
@@ -75992,7 +75989,7 @@
         <v>225</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F48" s="5" t="s">
         <v>184</v>
@@ -76024,7 +76021,7 @@
         <v>225</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>184</v>
@@ -76056,7 +76053,7 @@
         <v>225</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F50" s="5" t="s">
         <v>184</v>
@@ -76088,7 +76085,7 @@
         <v>225</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F51" s="5" t="s">
         <v>184</v>
@@ -76120,7 +76117,7 @@
         <v>225</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F52" s="5" t="s">
         <v>184</v>
@@ -76152,7 +76149,7 @@
         <v>225</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F53" s="5" t="s">
         <v>184</v>
@@ -76184,7 +76181,7 @@
         <v>225</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F54" s="5" t="s">
         <v>184</v>
@@ -76216,7 +76213,7 @@
         <v>225</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F55" s="5" t="s">
         <v>184</v>
@@ -77657,7 +77654,7 @@
       <c r="B31" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="10" t="s">
         <v>442</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -77677,7 +77674,7 @@
       <c r="B32" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="C32" s="11" t="s">
+      <c r="C32" s="10" t="s">
         <v>447</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -77697,7 +77694,7 @@
       <c r="B33" s="3" t="s">
         <v>450</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="11" t="s">
         <v>451</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -78065,22 +78062,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="15">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>504</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>505</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>365</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>361</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>354</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>357</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revised qty modifiers for stock report
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -73836,8 +73836,8 @@
       <c r="H55" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I55" s="8" t="s">
-        <v>200</v>
+      <c r="I55" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -73894,8 +73894,8 @@
       <c r="H57" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I57" s="8" t="s">
-        <v>252</v>
+      <c r="I57" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -76524,8 +76524,8 @@
       <c r="H58" s="11">
         <v>10.52</v>
       </c>
-      <c r="I58" s="8" t="s">
-        <v>200</v>
+      <c r="I58" s="6">
+        <v>1</v>
       </c>
       <c r="J58" s="4" t="s">
         <v>15</v>
@@ -76748,8 +76748,8 @@
       <c r="H65" s="11">
         <v>130.47999999999999</v>
       </c>
-      <c r="I65" s="8" t="s">
-        <v>252</v>
+      <c r="I65" s="6">
+        <v>1</v>
       </c>
       <c r="J65" s="4" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Amendments to toilet names on poster
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -8,7 +8,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="10"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -5030,13 +5030,13 @@
     <t>A-2-C1-F</t>
   </si>
   <si>
-    <t>Tower A Level 2 Cluster Toilet 1 (Female)</t>
+    <t>Tower A Level 2 A24 Cluster Toilet (Female)</t>
   </si>
   <si>
     <t>A-2-C1-M</t>
   </si>
   <si>
-    <t>Tower A Level 2 Cluster Toilet 1 (Male)</t>
+    <t>Tower A Level 2 A24 Cluster Toilet (Male)</t>
   </si>
   <si>
     <t>A-2-C2-F</t>
@@ -5045,13 +5045,13 @@
     <t>Retail</t>
   </si>
   <si>
-    <t>Tower A Level 2 Cluster 2 Toilet (Female)</t>
+    <t>Tower A Level 2 Retail Cluster Toilet (Female)</t>
   </si>
   <si>
     <t>A-2-C2-M</t>
   </si>
   <si>
-    <t>Tower A Level 2 Cluster 2 Toilet (Male)</t>
+    <t>Tower A Level 2 Retail Cluster Toilet (Male)</t>
   </si>
   <si>
     <t>B-1-EDP3-U1</t>

</xml_diff>

<commit_message>
Poster amendments and chat ID update
</commit_message>
<xml_diff>
--- a/Master Lists.xlsx
+++ b/Master Lists.xlsx
@@ -8,7 +8,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="16"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Item Master" sheetId="1" r:id="rId1"/>
@@ -5015,7 +5015,7 @@
     <t>Female</t>
   </si>
   <si>
-    <t>Tower A Level 1 Cluster Toilet(Female)</t>
+    <t>Tower A Level 1 Cluster Toilet (Female)</t>
   </si>
   <si>
     <t>A-1-CT-M</t>
@@ -5024,7 +5024,7 @@
     <t>Male</t>
   </si>
   <si>
-    <t>Tower A Level 1 Cluster Toilet(Male)</t>
+    <t>Tower A Level 1 Cluster Toilet (Male)</t>
   </si>
   <si>
     <t>A-2-C1-F</t>
@@ -81112,6 +81112,9 @@
       <c r="G14" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="I14" s="1">
+        <v>8961528240</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">

</xml_diff>